<commit_message>
feat(F-NAR-019): TREE-COL-030 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-COL-030.xlsx
+++ b/stories/arbres/TREE-COL-030.xlsx
@@ -1592,17 +1592,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Nina tape la vitre du doigt. Le verre fait toc, toc. Le ballon jaune sursaute dehors. Regardez ! Papa parle à maman, tout bas. Sa voix couvre le petit toc. Nina tape plus fort. Le ballon recule dans les branches. Non ! Elle arrête sa main. Elle pose le doigt sur le poignet de papa. Quand tu as fini, viens. Une seconde. Voilà, je t'écoute. Le rond s'est presque refermé. Dépêchons-nous, alors.</t>
+          <t>Nina tape la vitre du doigt. Le verre fait toc, toc. Le ballon jaune sursaute dehors. Regardez ! Papa chuchote à maman. Sa voix couvre le petit toc. Nina tape plus fort. Le ballon recule dans les branches. Non ! Elle arrête sa main. Elle pose le doigt sur le poignet de papa. Quand tu as fini, viens. Une seconde. Voilà, je t'écoute. Le rond s'est presque refermé. Dépêchons-nous, alors.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nina tape la vitre du doigt. Le verre fait toc, toc. Le ballon jaune sursaute dehors. Regardez ! Papa parle à maman, tout bas. Sa voix couvre le petit toc. Nina tape plus fort. Le ballon recule dans les branches. Non ! Elle arrête sa main. Elle pose le doigt sur le poignet de papa. Quand tu as fini, viens. Une seconde. Voilà, je t'écoute. Le rond s'est presque refermé. Dépêchons-nous, alors.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nina tape la vitre du doigt. Le verre fait toc, toc. Le ballon jaune sursaute dehors. Regardez ! Papa chuchote à maman. Sa voix couvre le petit toc. Nina tape plus fort. Le ballon recule dans les branches. Non ! Elle arrête sa main. Elle pose le doigt sur le poignet de papa. Quand tu as fini, viens. Une seconde. Voilà, je t'écoute. Le rond s'est presque refermé. Dépêchons-nous, alors.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Nina tape la vitre du doigt. Le verre fait toc, toc. Le ballon jaune sursaute dehors. Regardez ! Papa parle à maman, tout bas. Sa voix couvre le petit toc. Nina tape plus fort. Le ballon recule dans les branches. Non ! Elle arrête sa main. Elle pose le doigt sur le poignet de papa. Quand tu as fini, viens. Une seconde. Voilà, je t'écoute. Le rond s'est presque refermé. Dépêchons-nous, alors. [pause]</t>
+          <t>Nina tape la vitre du doigt. Le verre fait toc, toc. Le ballon jaune sursaute dehors. Regardez ! Papa chuchote à maman. Sa voix couvre le petit toc. Nina tape plus fort. Le ballon recule dans les branches. Non ! Elle arrête sa main. Elle pose le doigt sur le poignet de papa. Quand tu as fini, viens. Une seconde. Voilà, je t'écoute. Le rond s'est presque refermé. Dépêchons-nous, alors. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1740,7 +1740,7 @@
 narrateur|Le verre fait toc, toc.
 narrateur|Le ballon jaune sursaute dehors.
 enfant-f|Regardez !
-narrateur|Papa parle à maman, tout bas.
+narrateur|Papa chuchote à maman.
 narrateur|Sa voix couvre le petit toc.
 narrateur|Nina tape plus fort.
 narrateur|Le ballon recule dans les branches.
@@ -8532,17 +8532,17 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Une feuille de romarin flotte dans la tasse. À toi, Nina. Nous t'écoutons. J'ai gardé la tasse. Papa poussait. Merci d'avoir gardé la tasse. La tasse penche, comme le bâton. Le rond sent le cacao, tout contre le nez.</t>
+          <t>Une feuille de romarin flotte dans la tasse. À toi, Nina. Nous t'écoutons. J'ai gardé la tasse. Papa poussait. Merci d'avoir gardé la tasse. La tasse penche, comme le bâton. Le rond sent le cacao, contre le nez.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Une feuille de romarin flotte dans la tasse. À toi, Nina. Nous t'écoutons. J'ai gardé la tasse. Papa poussait. Merci d'avoir gardé la tasse. La tasse penche, comme le bâton. Le rond sent le cacao, tout contre le nez.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Une feuille de romarin flotte dans la tasse. À toi, Nina. Nous t'écoutons. J'ai gardé la tasse. Papa poussait. Merci d'avoir gardé la tasse. La tasse penche, comme le bâton. Le rond sent le cacao, contre le nez.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Une feuille de romarin flotte dans la tasse. À toi, Nina. Nous t'écoutons. J'ai gardé la tasse. Papa poussait. Merci d'avoir gardé la tasse. La tasse penche, comme le bâton. Le rond sent le cacao, tout contre le nez.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Une feuille de romarin flotte dans la tasse. À toi, Nina. Nous t'écoutons. J'ai gardé la tasse. Papa poussait. Merci d'avoir gardé la tasse. La tasse penche, comme le bâton. Le rond sent le cacao, contre le nez.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr"/>
@@ -8683,7 +8683,7 @@
 enfant-f|Papa poussait.
 papa|Merci d'avoir gardé la tasse.
 narrateur|La tasse penche, comme le bâton.
-narrateur|Le rond sent le cacao, tout contre le nez.</t>
+narrateur|Le rond sent le cacao, contre le nez.</t>
         </is>
       </c>
       <c r="AX41" t="inlineStr">
@@ -10395,17 +10395,17 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>La tasse reflète la fenêtre, toute ronde. À toi, Nina. Nous t'écoutons. On n'a pas marché dans l'eau. Merci d'avoir laissé l'eau se taire. La tasse reflète le ciel, près de l'eau. Le rond est un miroir, comme l'eau.</t>
+          <t>La tasse reflète la fenêtre, ronde. À toi, Nina. Nous t'écoutons. On n'a pas marché dans l'eau. Merci d'avoir laissé l'eau se taire. La tasse reflète le ciel, près de l'eau. Le rond est un miroir, comme l'eau.</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La tasse reflète la fenêtre, toute ronde. À toi, Nina. Nous t'écoutons. On n'a pas marché dans l'eau. Merci d'avoir laissé l'eau se taire. La tasse reflète le ciel, près de l'eau. Le rond est un miroir, comme l'eau.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La tasse reflète la fenêtre, ronde. À toi, Nina. Nous t'écoutons. On n'a pas marché dans l'eau. Merci d'avoir laissé l'eau se taire. La tasse reflète le ciel, près de l'eau. Le rond est un miroir, comme l'eau.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La tasse reflète la fenêtre, toute ronde. À toi, Nina. Nous t'écoutons. On n'a pas marché dans l'eau. Merci d'avoir laissé l'eau se taire. La tasse reflète le ciel, près de l'eau. Le rond est un miroir, comme l'eau.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La tasse reflète la fenêtre, ronde. À toi, Nina. Nous t'écoutons. On n'a pas marché dans l'eau. Merci d'avoir laissé l'eau se taire. La tasse reflète le ciel, près de l'eau. Le rond est un miroir, comme l'eau.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr"/>
@@ -10539,7 +10539,7 @@
       </c>
       <c r="AW51" t="inlineStr">
         <is>
-          <t>narrateur|La tasse reflète la fenêtre, toute ronde.
+          <t>narrateur|La tasse reflète la fenêtre, ronde.
 maman|À toi, Nina.
 maman|Nous t'écoutons.
 enfant-f|On n'a pas marché dans l'eau.
@@ -15637,17 +15637,17 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>Maman souffle sur le dessin, tout léger. À toi, Nina. Nous t'écoutons. L'eau s'est tue. Le crayon aussi. Merci d'avoir distingué le vrai. Le dessin attend, pendant que l'eau se tait. Nina efface le dessin, garde le petit rond.</t>
+          <t>Maman souffle sur le dessin, un peu. À toi, Nina. Nous t'écoutons. L'eau s'est tue. Le crayon aussi. Merci d'avoir montré le vrai. Le dessin attend, pendant que l'eau se tait. Nina efface le dessin, garde le petit rond.</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Maman souffle sur le dessin, tout léger. À toi, Nina. Nous t'écoutons. L'eau s'est tue. Le crayon aussi. Merci d'avoir distingué le vrai. Le dessin attend, pendant que l'eau se tait. Nina efface le dessin, garde le petit rond.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Maman souffle sur le dessin, un peu. À toi, Nina. Nous t'écoutons. L'eau s'est tue. Le crayon aussi. Merci d'avoir montré le vrai. Le dessin attend, pendant que l'eau se tait. Nina efface le dessin, garde le petit rond.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Maman souffle sur le dessin, tout léger. À toi, Nina. Nous t'écoutons. L'eau s'est tue. Le crayon aussi. Merci d'avoir distingué le vrai. Le dessin attend, pendant que l'eau se tait. Nina efface le dessin, garde le petit rond.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Maman souffle sur le dessin, un peu. À toi, Nina. Nous t'écoutons. L'eau s'est tue. Le crayon aussi. Merci d'avoir montré le vrai. Le dessin attend, pendant que l'eau se tait. Nina efface le dessin, garde le petit rond.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr"/>
@@ -15781,12 +15781,12 @@
       </c>
       <c r="AW79" t="inlineStr">
         <is>
-          <t>narrateur|Maman souffle sur le dessin, tout léger.
+          <t>narrateur|Maman souffle sur le dessin, un peu.
 maman|À toi, Nina.
 maman|Nous t'écoutons.
 enfant-f|L'eau s'est tue.
 enfant-f|Le crayon aussi.
-papa|Merci d'avoir distingué le vrai.
+papa|Merci d'avoir montré le vrai.
 narrateur|Le dessin attend, pendant que l'eau se tait.
 narrateur|Nina efface le dessin, garde le petit rond.</t>
         </is>
@@ -16395,17 +16395,17 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Le crayon pointe vers le jardin, oublié. À toi, Nina. Nous t'écoutons. J'ai pincé le gond. Le dessin restait. Le gond et le crayon se ressemblent, un peu. Le crayon a laissé un gond minuscule, au rebord. Le rond cadre le gond, tout petit.</t>
+          <t>Le crayon pointe vers le jardin, oublié. À toi, Nina. Nous t'écoutons. J'ai pincé le gond. Le dessin restait. Le gond et le crayon se ressemblent, un peu. Le crayon a laissé un gond minuscule, au rebord. Le rond cadre le gond, minuscule.</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le crayon pointe vers le jardin, oublié. À toi, Nina. Nous t'écoutons. J'ai pincé le gond. Le dessin restait. Le gond et le crayon se ressemblent, un peu. Le crayon a laissé un gond minuscule, au rebord. Le rond cadre le gond, tout petit.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le crayon pointe vers le jardin, oublié. À toi, Nina. Nous t'écoutons. J'ai pincé le gond. Le dessin restait. Le gond et le crayon se ressemblent, un peu. Le crayon a laissé un gond minuscule, au rebord. Le rond cadre le gond, minuscule.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le crayon pointe vers le jardin, oublié. À toi, Nina. Nous t'écoutons. J'ai pincé le gond. Le dessin restait. Le gond et le crayon se ressemblent, un peu. Le crayon a laissé un gond minuscule, au rebord. Le rond cadre le gond, tout petit.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le crayon pointe vers le jardin, oublié. À toi, Nina. Nous t'écoutons. J'ai pincé le gond. Le dessin restait. Le gond et le crayon se ressemblent, un peu. Le crayon a laissé un gond minuscule, au rebord. Le rond cadre le gond, minuscule.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr"/>
@@ -16546,7 +16546,7 @@
 enfant-f|Le dessin restait.
 papa|Le gond et le crayon se ressemblent, un peu.
 narrateur|Le crayon a laissé un gond minuscule, au rebord.
-narrateur|Le rond cadre le gond, tout petit.</t>
+narrateur|Le rond cadre le gond, minuscule.</t>
         </is>
       </c>
       <c r="AX83" t="inlineStr">
@@ -17311,7 +17311,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17368,6 +17368,13 @@
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>